<commit_message>
Interpolation_integration script v2 started
Realized allignment to the global axis created downstream problems with triplicate merging, instead allignment to a time-of application axis will be implemented

Using this as an opportunity to start from scratch, creating a cleaner script-structure

also created som Excel-files for pig slurry lab data
</commit_message>
<xml_diff>
--- a/Field-trails/Cattle-Slurry 2025-10-28/DFC overview cattle.xlsx
+++ b/Field-trails/Cattle-Slurry 2025-10-28/DFC overview cattle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\Cattle-Slurry 2025-10-28\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9690856E-42E8-43AF-B914-386B4976EF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B749A9-66EF-470D-A60F-5B8B464E9C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>Comments</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>Q [L/s]</t>
+  </si>
+  <si>
+    <t>Δt [h]</t>
   </si>
 </sst>
 </file>
@@ -288,11 +291,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -593,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="57.21875" bestFit="1" customWidth="1"/>
@@ -602,11 +606,11 @@
     <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,25 +630,28 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>45958</v>
       </c>
@@ -663,28 +670,31 @@
       <c r="G2" s="3">
         <v>0.43611111111111112</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
         <v>0.4513888888888889</v>
       </c>
-      <c r="I2">
-        <f>(F2^0.5)*$L$2</f>
+      <c r="J2">
+        <f>(F2^0.5)*$M$2</f>
         <v>34.36277055186325</v>
       </c>
-      <c r="J2" s="3">
-        <f>H2-G2</f>
+      <c r="K2" s="3">
+        <f>I2-G2</f>
         <v>1.5277777777777779E-2</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>3</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>23</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -703,11 +713,15 @@
       <c r="G3" s="3">
         <v>0.44166666666666665</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="4">
+        <f>H2+(8/60)</f>
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="I3" s="3">
         <v>0.45694444444444443</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -726,15 +740,19 @@
       <c r="G4" s="3">
         <v>0.44722222222222202</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
+        <f t="shared" ref="H4:H13" si="0">H3+(8/60)</f>
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="I4" s="3">
         <v>0.46250000000000002</v>
       </c>
-      <c r="I4">
-        <f t="shared" ref="I3:I13" si="0">(F4^0.5)*$L$2</f>
+      <c r="J4">
+        <f>(F4^0.5)*$M$2</f>
         <v>34.36277055186325</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -753,11 +771,15 @@
       <c r="G5" s="3">
         <v>0.452777777777778</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="4">
+        <f t="shared" si="0"/>
+        <v>0.4</v>
+      </c>
+      <c r="I5" s="3">
         <v>0.468055555555556</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -776,15 +798,19 @@
       <c r="G6" s="3">
         <v>0.45833333333333298</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="4">
+        <f t="shared" si="0"/>
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="I6" s="3">
         <v>0.47361111111111098</v>
       </c>
-      <c r="I6">
-        <f t="shared" si="0"/>
+      <c r="J6">
+        <f>(F6^0.5)*$M$2</f>
         <v>33.634803403617511</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C7">
         <v>12</v>
       </c>
@@ -800,15 +826,19 @@
       <c r="G7" s="3">
         <v>0.46388888888888902</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="4">
+        <f t="shared" si="0"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="I7" s="3">
         <v>0.47916666666666702</v>
       </c>
-      <c r="I7">
-        <f t="shared" si="0"/>
+      <c r="J7">
+        <f>(F7^0.5)*$M$2</f>
         <v>34.139420030223128</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -827,15 +857,19 @@
       <c r="G8" s="3">
         <v>0.469444444444444</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="4">
+        <f t="shared" si="0"/>
+        <v>0.79999999999999993</v>
+      </c>
+      <c r="I8" s="3">
         <v>0.484722222222222</v>
       </c>
-      <c r="I8">
-        <f t="shared" si="0"/>
+      <c r="J8">
+        <f>(F8^0.5)*$M$2</f>
         <v>33.848190498164001</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -854,15 +888,19 @@
       <c r="G9" s="3">
         <v>0.47499999999999998</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="4">
+        <f t="shared" si="0"/>
+        <v>0.93333333333333324</v>
+      </c>
+      <c r="I9" s="3">
         <v>0.49027777777777798</v>
       </c>
-      <c r="I9">
-        <f t="shared" si="0"/>
+      <c r="J9">
+        <f>(F9^0.5)*$M$2</f>
         <v>34.415112959279966</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -881,15 +919,19 @@
       <c r="G10" s="3">
         <v>0.48055555555555501</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="4">
+        <f t="shared" si="0"/>
+        <v>1.0666666666666667</v>
+      </c>
+      <c r="I10" s="3">
         <v>0.49583333333333302</v>
       </c>
-      <c r="I10">
-        <f t="shared" si="0"/>
+      <c r="J10">
+        <f>(F10^0.5)*$M$2</f>
         <v>34.375863625514924</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C11">
         <v>16</v>
       </c>
@@ -905,11 +947,15 @@
       <c r="G11" s="3">
         <v>0.48611111111111099</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="4">
+        <f t="shared" si="0"/>
+        <v>1.2</v>
+      </c>
+      <c r="I11" s="3">
         <v>0.50138888888888899</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C12">
         <v>17</v>
       </c>
@@ -925,15 +971,19 @@
       <c r="G12" s="3">
         <v>0.49166666666666697</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="4">
+        <f t="shared" si="0"/>
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="I12" s="3">
         <v>0.50694444444444398</v>
       </c>
-      <c r="I12">
-        <f t="shared" si="0"/>
+      <c r="J12">
+        <f>(F12^0.5)*$M$2</f>
         <v>34.139420030223128</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C13">
         <v>18</v>
       </c>
@@ -949,11 +999,15 @@
       <c r="G13" s="3">
         <v>0.49722222222222201</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="4">
+        <f t="shared" si="0"/>
+        <v>1.4666666666666666</v>
+      </c>
+      <c r="I13" s="3">
         <v>0.51249999999999996</v>
       </c>
-      <c r="I13">
-        <f t="shared" si="0"/>
+      <c r="J13">
+        <f>(F13^0.5)*$M$2</f>
         <v>33.621421742692561</v>
       </c>
     </row>

</xml_diff>